<commit_message>
Update example test file CFDataBars
Update reference test file for example CFDataBars. After style
infrastructure switch, the styles part is saved differently. No
semantic change to the styles part.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBars.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBars.xlsx
@@ -37,61 +37,52 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -515,7 +506,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38d9e5d3-73a7-4e18-b3b9-aa1b26e4cc06}</x14:id>
+          <x14:id>{5d30806a-f8bc-486c-b2cc-9391932bac5e}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -529,7 +520,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0671ebad-2a52-43f6-a3a9-585018af6f01}</x14:id>
+          <x14:id>{b4c702ec-4f90-4f87-9d08-505c18166b58}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -543,7 +534,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0b10551c-b4e0-4975-ac10-c045e09df4bf}</x14:id>
+          <x14:id>{cddaad48-b1b6-46a9-8ef3-330adecf7baa}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -557,7 +548,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49ad88bb-d5a9-4684-afcc-8033d8d051eb}</x14:id>
+          <x14:id>{23068bd3-f630-47d0-9a83-01fbfff8e7e4}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -571,7 +562,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93055e58-8649-4a74-9a8e-1e4036062ece}</x14:id>
+          <x14:id>{ed6d6dc8-01ec-425e-98c2-bd5aaef133b1}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -585,7 +576,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{01b3b3bb-243e-4add-ae5b-fd208d5e5960}</x14:id>
+          <x14:id>{638c99e3-ba9d-49e5-84d6-7be58eaf1c9f}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -599,7 +590,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38d9e5d3-73a7-4e18-b3b9-aa1b26e4cc06}">
+          <x14:cfRule type="dataBar" id="{5d30806a-f8bc-486c-b2cc-9391932bac5e}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -610,7 +601,7 @@
           <xm:sqref>A2:A6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0671ebad-2a52-43f6-a3a9-585018af6f01}">
+          <x14:cfRule type="dataBar" id="{b4c702ec-4f90-4f87-9d08-505c18166b58}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -625,7 +616,7 @@
           <xm:sqref>B2:B6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0b10551c-b4e0-4975-ac10-c045e09df4bf}">
+          <x14:cfRule type="dataBar" id="{cddaad48-b1b6-46a9-8ef3-330adecf7baa}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -640,7 +631,7 @@
           <xm:sqref>C2:C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49ad88bb-d5a9-4684-afcc-8033d8d051eb}">
+          <x14:cfRule type="dataBar" id="{23068bd3-f630-47d0-9a83-01fbfff8e7e4}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>50</xm:f>
@@ -655,7 +646,7 @@
           <xm:sqref>D2:D6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93055e58-8649-4a74-9a8e-1e4036062ece}">
+          <x14:cfRule type="dataBar" id="{ed6d6dc8-01ec-425e-98c2-bd5aaef133b1}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>-SUM($A$2:$E$2)</xm:f>
@@ -670,7 +661,7 @@
           <xm:sqref>E2:E6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{01b3b3bb-243e-4add-ae5b-fd208d5e5960}">
+          <x14:cfRule type="dataBar" id="{638c99e3-ba9d-49e5-84d6-7be58eaf1c9f}">
             <x14:dataBar minLength="0" maxLength="100" showValue="1" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>30</xm:f>

</xml_diff>